<commit_message>
Updates scenario prices and gas limits
Updates the scenario pricing mechanism to dynamically read and apply prices for LNG, piped gas, and various technologies (solarPV, windon, windoff, Batteries) based on the window start year.
This enhancement enables more accurate modeling of future energy scenarios by incorporating scenario-specific price projections.

Also, decreases the maximum value for 'Piped Gas' commodity over time with a 4.052% yearly decrease from 2024 to 2050.
</commit_message>
<xml_diff>
--- a/scenario_specific_data.xlsx
+++ b/scenario_specific_data.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28827"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28925"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\maxoi\GitHub\urbs-extension\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C11A7899-3799-4720-A70E-9758303E01D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{214930D9-C62F-4C29-88E9-B7A761B5F755}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-5445" windowWidth="38640" windowHeight="21120" xr2:uid="{135E7A19-983F-4672-B1BC-B86D20613CB6}"/>
+    <workbookView xWindow="67080" yWindow="-1935" windowWidth="29040" windowHeight="17520" activeTab="1" xr2:uid="{135E7A19-983F-4672-B1BC-B86D20613CB6}"/>
   </bookViews>
   <sheets>
     <sheet name="import_prices" sheetId="1" r:id="rId1"/>
@@ -18,6 +18,7 @@
     <sheet name="piped_gas_prices" sheetId="2" r:id="rId3"/>
     <sheet name="lng_prices" sheetId="3" r:id="rId4"/>
     <sheet name="piped_gas_trajectory" sheetId="4" r:id="rId5"/>
+    <sheet name="elec_demand" sheetId="6" r:id="rId6"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -40,7 +41,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="74" uniqueCount="68">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="81" uniqueCount="74">
   <si>
     <t>Stf</t>
   </si>
@@ -245,6 +246,24 @@
   <si>
     <t>manufacturing_EU27_Batteries_2049</t>
   </si>
+  <si>
+    <t>elec_dem_2024</t>
+  </si>
+  <si>
+    <t>elec_dem_2029</t>
+  </si>
+  <si>
+    <t>elec_dem_2034</t>
+  </si>
+  <si>
+    <t>elec_dem_2039</t>
+  </si>
+  <si>
+    <t>elec_dem_2044</t>
+  </si>
+  <si>
+    <t>elec_dem_2049</t>
+  </si>
 </sst>
 </file>
 
@@ -291,10 +310,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="top"/>
+    </xf>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -3792,35 +3814,15 @@
       <c r="B2">
         <v>250240</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
       <c r="H2">
         <v>1052044.8400000001</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
       <c r="N2">
         <v>1775265.6417320003</v>
       </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
       <c r="T2">
-        <v>90210</v>
-      </c>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2"/>
+        <v>280439.83</v>
+      </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -3829,35 +3831,15 @@
       <c r="B3">
         <v>246486.39999999999</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
       <c r="H3">
         <v>1042480.7960000001</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
       <c r="N3">
         <v>1722922.372057667</v>
       </c>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
       <c r="T3">
-        <v>88856.85</v>
-      </c>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
+        <v>274754.90999999997</v>
+      </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -3866,35 +3848,15 @@
       <c r="B4">
         <v>242789.10399999999</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
       <c r="H4">
         <v>1032916.7520000001</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
       <c r="N4">
         <v>1670579.1023833335</v>
       </c>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
       <c r="T4">
-        <v>87523</v>
-      </c>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
+        <v>269179.44</v>
+      </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -3903,35 +3865,15 @@
       <c r="B5">
         <v>239147.26740000001</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
       <c r="H5">
         <v>1023352.708</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
       <c r="N5">
         <v>1618235.832709</v>
       </c>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
       <c r="T5">
-        <v>86209.15</v>
-      </c>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
+        <v>263711.78000000003</v>
+      </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -3940,35 +3882,15 @@
       <c r="B6">
         <v>235560.05840000001</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
       <c r="H6">
         <v>1013788.6639999999</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
       <c r="N6">
         <v>1565892.5630346665</v>
       </c>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
       <c r="T6">
-        <v>84915.01</v>
-      </c>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+        <v>258350.32</v>
+      </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -3980,40 +3902,24 @@
       <c r="C7">
         <v>232026.65760000001</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
       <c r="H7">
         <v>1004224.62</v>
       </c>
       <c r="I7">
         <v>1004224.62</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
       <c r="N7">
         <v>1513549.293360333</v>
       </c>
       <c r="O7">
         <v>1513549.293360333</v>
       </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
       <c r="T7">
-        <v>83640.289999999994</v>
+        <v>253093.46</v>
       </c>
       <c r="U7">
-        <v>83640.289999999994</v>
-      </c>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
+        <v>253093.46</v>
+      </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -4023,42 +3929,26 @@
         <v>228546.25769999999</v>
       </c>
       <c r="C8">
-        <v>228546.25769999999</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+        <v>278546.25770000002</v>
+      </c>
       <c r="H8">
         <v>994660.57600000012</v>
       </c>
       <c r="I8">
-        <v>994660.57600000012</v>
-      </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+        <v>1044660.576</v>
+      </c>
       <c r="N8">
         <v>1461206.0236859999</v>
       </c>
       <c r="O8">
-        <v>1461206.0236859999</v>
-      </c>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
+        <v>1511206.024</v>
+      </c>
       <c r="T8">
-        <v>82384.69</v>
+        <v>247939.65</v>
       </c>
       <c r="U8">
-        <v>82384.69</v>
-      </c>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
+        <v>297939.65000000002</v>
+      </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -4068,42 +3958,26 @@
         <v>225118.0638</v>
       </c>
       <c r="C9">
-        <v>225118.0638</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+        <v>275118.0638</v>
+      </c>
       <c r="H9">
         <v>992747.76720000012</v>
       </c>
       <c r="I9">
-        <v>992747.76720000012</v>
-      </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+        <v>1042747.7672</v>
+      </c>
       <c r="N9">
         <v>1444015.15599508</v>
       </c>
       <c r="O9">
-        <v>1444015.15599508</v>
-      </c>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
+        <v>1494015.156</v>
+      </c>
       <c r="T9">
-        <v>81147.92</v>
+        <v>242887.37</v>
       </c>
       <c r="U9">
-        <v>81147.92</v>
-      </c>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
-      <c r="Y9" s="2"/>
+        <v>292887.37</v>
+      </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -4113,42 +3987,26 @@
         <v>221741.2929</v>
       </c>
       <c r="C10">
-        <v>221741.2929</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+        <v>271741.2929</v>
+      </c>
       <c r="H10">
         <v>990834.9584</v>
       </c>
       <c r="I10">
-        <v>990834.9584</v>
-      </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+        <v>1040834.9584</v>
+      </c>
       <c r="N10">
         <v>1426824.2883041599</v>
       </c>
       <c r="O10">
-        <v>1426824.2883041599</v>
-      </c>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
+        <v>1476824.2879999999</v>
+      </c>
       <c r="T10">
-        <v>79929.7</v>
+        <v>237935.1</v>
       </c>
       <c r="U10">
-        <v>79929.7</v>
-      </c>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-      <c r="Y10" s="2"/>
+        <v>287935.09999999998</v>
+      </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -4158,42 +4016,26 @@
         <v>218415.1735</v>
       </c>
       <c r="C11">
-        <v>218415.1735</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+        <v>268415.17349999998</v>
+      </c>
       <c r="H11">
         <v>988922.1496</v>
       </c>
       <c r="I11">
-        <v>988922.1496</v>
-      </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+        <v>1038922.1496</v>
+      </c>
       <c r="N11">
         <v>1409633.42061324</v>
       </c>
       <c r="O11">
-        <v>1409633.42061324</v>
-      </c>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
+        <v>1459633.4210000001</v>
+      </c>
       <c r="T11">
-        <v>78729.759999999995</v>
+        <v>233081.4</v>
       </c>
       <c r="U11">
-        <v>78729.759999999995</v>
-      </c>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
+        <v>283081.40000000002</v>
+      </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -4203,50 +4045,38 @@
         <v>215138.94589999999</v>
       </c>
       <c r="C12">
-        <v>215138.94589999999</v>
+        <v>265138.94589999999</v>
       </c>
       <c r="D12">
         <v>215138.94589999999</v>
       </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
       <c r="H12">
         <v>987009.34079999989</v>
       </c>
       <c r="I12">
-        <v>987009.34079999989</v>
-      </c>
-      <c r="J12">
-        <v>987009.34079999989</v>
-      </c>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+        <v>1037009.3408</v>
+      </c>
+      <c r="J12" s="4">
+        <v>987009.34</v>
+      </c>
       <c r="N12">
         <v>1392442.5529223196</v>
       </c>
       <c r="O12">
-        <v>1392442.5529223196</v>
+        <v>1442442.5530000001</v>
       </c>
       <c r="P12">
         <v>1392442.5529223196</v>
       </c>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
       <c r="T12">
-        <v>77547.820000000007</v>
+        <v>228324.82</v>
       </c>
       <c r="U12">
-        <v>77547.820000000007</v>
+        <v>278324.82</v>
       </c>
       <c r="V12">
-        <v>77547.820000000007</v>
-      </c>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
+        <v>228324.82</v>
+      </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -4256,50 +4086,38 @@
         <v>211911.86170000001</v>
       </c>
       <c r="C13">
-        <v>211911.86170000001</v>
+        <v>261911.86170000001</v>
       </c>
       <c r="D13">
-        <v>211911.86170000001</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+        <v>317867.79255000001</v>
+      </c>
       <c r="H13">
         <v>985096.53199999989</v>
       </c>
       <c r="I13">
-        <v>985096.53199999989</v>
-      </c>
-      <c r="J13">
-        <v>985096.53199999989</v>
-      </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+        <v>1035096.532</v>
+      </c>
+      <c r="J13" s="4">
+        <v>1477644.798</v>
+      </c>
       <c r="N13">
         <v>1375251.6852313997</v>
       </c>
       <c r="O13">
-        <v>1375251.6852313997</v>
+        <v>1425251.6850000001</v>
       </c>
       <c r="P13">
-        <v>1375251.6852313997</v>
-      </c>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
+        <v>2062877.5275000001</v>
+      </c>
       <c r="T13">
-        <v>76383.600000000006</v>
+        <v>223663.91</v>
       </c>
       <c r="U13">
-        <v>76383.600000000006</v>
+        <v>273663.90999999997</v>
       </c>
       <c r="V13">
-        <v>76383.600000000006</v>
-      </c>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-      <c r="Y13" s="2"/>
+        <v>335495.86499999999</v>
+      </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -4309,50 +4127,38 @@
         <v>208733.1838</v>
       </c>
       <c r="C14">
-        <v>208733.1838</v>
+        <v>258733.1838</v>
       </c>
       <c r="D14">
-        <v>208733.1838</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+        <v>313099.7757</v>
+      </c>
       <c r="H14">
         <v>983183.72319999977</v>
       </c>
       <c r="I14">
-        <v>983183.72319999977</v>
-      </c>
-      <c r="J14">
-        <v>983183.72319999977</v>
-      </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+        <v>1033183.7232</v>
+      </c>
+      <c r="J14" s="4">
+        <v>1474775.5848000001</v>
+      </c>
       <c r="N14">
         <v>1358060.8175404796</v>
       </c>
       <c r="O14">
-        <v>1358060.8175404796</v>
+        <v>1408060.818</v>
       </c>
       <c r="P14">
-        <v>1358060.8175404796</v>
-      </c>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
+        <v>2037091.227</v>
+      </c>
       <c r="T14">
-        <v>75236.84</v>
+        <v>219097.32</v>
       </c>
       <c r="U14">
-        <v>75236.84</v>
+        <v>269097.32</v>
       </c>
       <c r="V14">
-        <v>75236.84</v>
-      </c>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-      <c r="Y14" s="2"/>
+        <v>328645.98</v>
+      </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -4362,50 +4168,38 @@
         <v>205602.18599999999</v>
       </c>
       <c r="C15">
-        <v>205602.18599999999</v>
+        <v>255602.18599999999</v>
       </c>
       <c r="D15">
-        <v>205602.18599999999</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+        <v>308403.27899999998</v>
+      </c>
       <c r="H15">
         <v>981270.91439999978</v>
       </c>
       <c r="I15">
-        <v>981270.91439999978</v>
-      </c>
-      <c r="J15">
-        <v>981270.91439999978</v>
-      </c>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+        <v>1031270.9144</v>
+      </c>
+      <c r="J15" s="4">
+        <v>1471906.3716</v>
+      </c>
       <c r="N15">
         <v>1340869.9498495597</v>
       </c>
       <c r="O15">
-        <v>1340869.9498495597</v>
+        <v>1390869.95</v>
       </c>
       <c r="P15">
-        <v>1340869.9498495597</v>
-      </c>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+        <v>2011304.925</v>
+      </c>
       <c r="T15">
-        <v>74107.289999999994</v>
+        <v>214623.65</v>
       </c>
       <c r="U15">
-        <v>74107.289999999994</v>
+        <v>264623.65000000002</v>
       </c>
       <c r="V15">
-        <v>74107.289999999994</v>
-      </c>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
+        <v>321935.47499999998</v>
+      </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16">
@@ -4415,50 +4209,38 @@
         <v>202518.1532</v>
       </c>
       <c r="C16">
-        <v>202518.1532</v>
+        <v>252518.1532</v>
       </c>
       <c r="D16">
-        <v>202518.1532</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+        <v>303777.22979999997</v>
+      </c>
       <c r="H16">
         <v>979358.10559999966</v>
       </c>
       <c r="I16">
-        <v>979358.10559999966</v>
-      </c>
-      <c r="J16">
-        <v>979358.10559999966</v>
-      </c>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
+        <v>1029358.1056</v>
+      </c>
+      <c r="J16" s="4">
+        <v>1469037.1584000001</v>
+      </c>
       <c r="N16">
         <v>1323679.0821586396</v>
       </c>
       <c r="O16">
-        <v>1323679.0821586396</v>
+        <v>1373679.0819999999</v>
       </c>
       <c r="P16">
-        <v>1323679.0821586396</v>
-      </c>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
+        <v>1985518.6229999999</v>
+      </c>
       <c r="T16">
-        <v>72994.679999999993</v>
+        <v>210241.6</v>
       </c>
       <c r="U16">
-        <v>72994.679999999993</v>
+        <v>260241.6</v>
       </c>
       <c r="V16">
-        <v>72994.679999999993</v>
-      </c>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
-      <c r="Y16" s="2"/>
+        <v>315362.40000000002</v>
+      </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17">
@@ -4468,58 +4250,50 @@
         <v>199480.38089999999</v>
       </c>
       <c r="C17">
-        <v>199480.38089999999</v>
+        <v>249480.38089999999</v>
       </c>
       <c r="D17">
-        <v>199480.38089999999</v>
+        <v>299220.57134999998</v>
       </c>
       <c r="E17">
-        <v>199480.38089999999</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+        <v>299220.57134999998</v>
+      </c>
       <c r="H17">
         <v>977445.29679999966</v>
       </c>
       <c r="I17">
-        <v>977445.29679999966</v>
-      </c>
-      <c r="J17">
-        <v>977445.29679999966</v>
-      </c>
-      <c r="K17">
-        <v>977445.29679999966</v>
-      </c>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+        <v>1027445.2968</v>
+      </c>
+      <c r="J17" s="4">
+        <v>1466167.9452</v>
+      </c>
+      <c r="K17" s="4">
+        <v>1466167.9452</v>
+      </c>
       <c r="N17">
         <v>1306488.2144677194</v>
       </c>
       <c r="O17">
-        <v>1306488.2144677194</v>
+        <v>1356488.2139999999</v>
       </c>
       <c r="P17">
-        <v>1306488.2144677194</v>
+        <v>1959732.321</v>
       </c>
       <c r="Q17">
-        <v>1306488.2144677194</v>
-      </c>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
+        <v>1959732.321</v>
+      </c>
       <c r="T17">
-        <v>71898.759999999995</v>
+        <v>205949.84</v>
       </c>
       <c r="U17">
-        <v>71898.759999999995</v>
+        <v>255949.84</v>
       </c>
       <c r="V17">
-        <v>71898.759999999995</v>
+        <v>308924.76</v>
       </c>
       <c r="W17">
-        <v>71898.759999999995</v>
-      </c>
-      <c r="X17" s="2"/>
-      <c r="Y17" s="2"/>
+        <v>308924.76</v>
+      </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A18">
@@ -4529,58 +4303,50 @@
         <v>196488.1752</v>
       </c>
       <c r="C18">
-        <v>196488.1752</v>
+        <v>246488.1752</v>
       </c>
       <c r="D18">
-        <v>196488.1752</v>
+        <v>294732.26280000003</v>
       </c>
       <c r="E18">
-        <v>196488.1752</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+        <v>294732.26280000003</v>
+      </c>
       <c r="H18">
         <v>975532.48799999955</v>
       </c>
       <c r="I18">
-        <v>975532.48799999955</v>
-      </c>
-      <c r="J18">
-        <v>975532.48799999955</v>
-      </c>
-      <c r="K18">
-        <v>975532.48799999955</v>
-      </c>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
+        <v>1025532.488</v>
+      </c>
+      <c r="J18" s="4">
+        <v>1463298.7320000001</v>
+      </c>
+      <c r="K18" s="4">
+        <v>1463298.7320000001</v>
+      </c>
       <c r="N18">
         <v>1288027.7959324</v>
       </c>
       <c r="O18">
-        <v>1288027.7959324</v>
+        <v>1338027.7960000001</v>
       </c>
       <c r="P18">
-        <v>1288027.7959324</v>
+        <v>1932041.6939999999</v>
       </c>
       <c r="Q18">
-        <v>1288027.7959324</v>
-      </c>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
+        <v>1932041.6939999999</v>
+      </c>
       <c r="T18">
-        <v>70819.28</v>
+        <v>201747.12</v>
       </c>
       <c r="U18">
-        <v>70819.28</v>
+        <v>251747.12</v>
       </c>
       <c r="V18">
-        <v>70819.28</v>
+        <v>302620.68</v>
       </c>
       <c r="W18">
-        <v>70819.28</v>
-      </c>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
+        <v>302620.68</v>
+      </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19">
@@ -4590,58 +4356,50 @@
         <v>193540.85260000001</v>
       </c>
       <c r="C19">
-        <v>193540.85260000001</v>
+        <v>243540.85260000001</v>
       </c>
       <c r="D19">
-        <v>193540.85260000001</v>
+        <v>290311.27889999998</v>
       </c>
       <c r="E19">
-        <v>193540.85260000001</v>
-      </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+        <v>290311.27889999998</v>
+      </c>
       <c r="H19">
         <v>973619.67919999966</v>
       </c>
       <c r="I19">
-        <v>973619.67919999966</v>
-      </c>
-      <c r="J19">
-        <v>973619.67919999966</v>
-      </c>
-      <c r="K19">
-        <v>973619.67919999966</v>
-      </c>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
+        <v>1023619.6792</v>
+      </c>
+      <c r="J19" s="4">
+        <v>1460429.52</v>
+      </c>
+      <c r="K19" s="4">
+        <v>1460429.52</v>
+      </c>
       <c r="N19">
         <v>1288154.7510168403</v>
       </c>
       <c r="O19">
-        <v>1288154.7510168403</v>
+        <v>1338154.7509999999</v>
       </c>
       <c r="P19">
-        <v>1288154.7510168403</v>
+        <v>1932232.1265</v>
       </c>
       <c r="Q19">
-        <v>1288154.7510168403</v>
-      </c>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
+        <v>1932232.1265</v>
+      </c>
       <c r="T19">
-        <v>69755.990000000005</v>
+        <v>197632.19</v>
       </c>
       <c r="U19">
-        <v>69755.990000000005</v>
+        <v>247632.19</v>
       </c>
       <c r="V19">
-        <v>69755.990000000005</v>
+        <v>296448.28499999997</v>
       </c>
       <c r="W19">
-        <v>69755.990000000005</v>
-      </c>
-      <c r="X19" s="2"/>
-      <c r="Y19" s="2"/>
+        <v>296448.28499999997</v>
+      </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20">
@@ -4651,58 +4409,50 @@
         <v>190637.73980000001</v>
       </c>
       <c r="C20">
-        <v>190637.73980000001</v>
+        <v>240637.73980000001</v>
       </c>
       <c r="D20">
-        <v>190637.73980000001</v>
+        <v>285956.60969999997</v>
       </c>
       <c r="E20">
-        <v>190637.73980000001</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+        <v>285956.60969999997</v>
+      </c>
       <c r="H20">
         <v>971706.87039999955</v>
       </c>
       <c r="I20">
-        <v>971706.87039999955</v>
-      </c>
-      <c r="J20">
-        <v>971706.87039999955</v>
-      </c>
-      <c r="K20">
-        <v>971706.87039999955</v>
-      </c>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+        <v>1021706.8704</v>
+      </c>
+      <c r="J20" s="4">
+        <v>1457560.3056000001</v>
+      </c>
+      <c r="K20" s="4">
+        <v>1457560.3056000001</v>
+      </c>
       <c r="N20">
         <v>1288281.7061012802</v>
       </c>
       <c r="O20">
-        <v>1288281.7061012802</v>
+        <v>1338281.706</v>
       </c>
       <c r="P20">
-        <v>1288281.7061012802</v>
+        <v>1932422.5589999999</v>
       </c>
       <c r="Q20">
-        <v>1288281.7061012802</v>
-      </c>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
+        <v>1932422.5589999999</v>
+      </c>
       <c r="T20">
-        <v>68708.649999999994</v>
+        <v>193603.83</v>
       </c>
       <c r="U20">
-        <v>68708.649999999994</v>
+        <v>243603.83</v>
       </c>
       <c r="V20">
-        <v>68708.649999999994</v>
+        <v>290405.745</v>
       </c>
       <c r="W20">
-        <v>68708.649999999994</v>
-      </c>
-      <c r="X20" s="2"/>
-      <c r="Y20" s="2"/>
+        <v>290405.745</v>
+      </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21">
@@ -4712,58 +4462,50 @@
         <v>187778.17370000001</v>
       </c>
       <c r="C21">
-        <v>187778.17370000001</v>
+        <v>237778.17370000001</v>
       </c>
       <c r="D21">
-        <v>187778.17370000001</v>
+        <v>281667.26055000001</v>
       </c>
       <c r="E21">
-        <v>187778.17370000001</v>
-      </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+        <v>281667.26055000001</v>
+      </c>
       <c r="H21">
         <v>969794.06159999955</v>
       </c>
       <c r="I21">
-        <v>969794.06159999955</v>
-      </c>
-      <c r="J21">
-        <v>969794.06159999955</v>
-      </c>
-      <c r="K21">
-        <v>969794.06159999955</v>
-      </c>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+        <v>1019794.0616</v>
+      </c>
+      <c r="J21" s="4">
+        <v>1454691.0924</v>
+      </c>
+      <c r="K21" s="4">
+        <v>1454691.0924</v>
+      </c>
       <c r="N21">
         <v>1288408.6611857202</v>
       </c>
       <c r="O21">
-        <v>1288408.6611857202</v>
+        <v>1338408.6610000001</v>
       </c>
       <c r="P21">
-        <v>1288408.6611857202</v>
+        <v>1932612.9915</v>
       </c>
       <c r="Q21">
-        <v>1288408.6611857202</v>
-      </c>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
+        <v>1932612.9915</v>
+      </c>
       <c r="T21">
-        <v>67677.02</v>
+        <v>189660.87</v>
       </c>
       <c r="U21">
-        <v>67677.02</v>
+        <v>239660.87</v>
       </c>
       <c r="V21">
-        <v>67677.02</v>
+        <v>284491.30499999999</v>
       </c>
       <c r="W21">
-        <v>67677.02</v>
-      </c>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
+        <v>284491.30499999999</v>
+      </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22">
@@ -4773,66 +4515,62 @@
         <v>184961.50109999999</v>
       </c>
       <c r="C22">
-        <v>184961.50109999999</v>
+        <v>234961.50109999999</v>
       </c>
       <c r="D22">
-        <v>184961.50109999999</v>
+        <v>277442.25164999999</v>
       </c>
       <c r="E22">
-        <v>184961.50109999999</v>
+        <v>277442.25164999999</v>
       </c>
       <c r="F22">
-        <v>184961.50109999999</v>
-      </c>
-      <c r="G22" s="2"/>
+        <v>277442.25164999999</v>
+      </c>
       <c r="H22">
         <v>967881.25279999943</v>
       </c>
       <c r="I22">
-        <v>967881.25279999943</v>
-      </c>
-      <c r="J22">
-        <v>967881.25279999943</v>
-      </c>
-      <c r="K22">
-        <v>967881.25279999943</v>
-      </c>
-      <c r="L22">
-        <v>967881.25279999943</v>
-      </c>
-      <c r="M22" s="2"/>
+        <v>1017881.2528</v>
+      </c>
+      <c r="J22" s="4">
+        <v>1451821.8792000001</v>
+      </c>
+      <c r="K22" s="4">
+        <v>1451821.8792000001</v>
+      </c>
+      <c r="L22" s="4">
+        <v>1451821.8792000001</v>
+      </c>
       <c r="N22">
         <v>1288535.6162701603</v>
       </c>
       <c r="O22">
-        <v>1288535.6162701603</v>
+        <v>1338535.6159999999</v>
       </c>
       <c r="P22">
-        <v>1288535.6162701603</v>
+        <v>1932803.4240000001</v>
       </c>
       <c r="Q22">
-        <v>1288535.6162701603</v>
+        <v>1932803.4240000001</v>
       </c>
       <c r="R22">
-        <v>1288535.6162701603</v>
-      </c>
-      <c r="S22" s="2"/>
+        <v>1932803.4240000001</v>
+      </c>
       <c r="T22">
-        <v>66660.86</v>
+        <v>185802.14</v>
       </c>
       <c r="U22">
-        <v>66660.86</v>
+        <v>235802.14</v>
       </c>
       <c r="V22">
-        <v>66660.86</v>
+        <v>278703.21000000002</v>
       </c>
       <c r="W22">
-        <v>66660.86</v>
+        <v>278703.21000000002</v>
       </c>
       <c r="X22">
-        <v>66660.86</v>
-      </c>
-      <c r="Y22" s="2"/>
+        <v>278703.21000000002</v>
+      </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23">
@@ -4842,66 +4580,62 @@
         <v>182187.07860000001</v>
       </c>
       <c r="C23">
-        <v>182187.07860000001</v>
+        <v>232187.07860000001</v>
       </c>
       <c r="D23">
-        <v>182187.07860000001</v>
+        <v>273280.6189</v>
       </c>
       <c r="E23">
-        <v>182187.07860000001</v>
+        <v>273280.6189</v>
       </c>
       <c r="F23">
-        <v>182187.07860000001</v>
-      </c>
-      <c r="G23" s="2"/>
+        <v>273280.6189</v>
+      </c>
       <c r="H23">
         <v>965968.44399999944</v>
       </c>
       <c r="I23">
-        <v>965968.44399999944</v>
-      </c>
-      <c r="J23">
-        <v>965968.44399999944</v>
-      </c>
-      <c r="K23">
-        <v>965968.44399999944</v>
-      </c>
-      <c r="L23">
-        <v>965968.44399999944</v>
-      </c>
-      <c r="M23" s="2"/>
+        <v>1015968.444</v>
+      </c>
+      <c r="J23" s="4">
+        <v>1448952.666</v>
+      </c>
+      <c r="K23" s="4">
+        <v>1448952.666</v>
+      </c>
+      <c r="L23" s="4">
+        <v>1448952.666</v>
+      </c>
       <c r="N23">
         <v>1288662.5713546001</v>
       </c>
       <c r="O23">
-        <v>1288662.5713546001</v>
+        <v>1338662.571</v>
       </c>
       <c r="P23">
-        <v>1288662.5713546001</v>
+        <v>1932993.8565</v>
       </c>
       <c r="Q23">
-        <v>1288662.5713546001</v>
+        <v>1932993.8565</v>
       </c>
       <c r="R23">
-        <v>1288662.5713546001</v>
-      </c>
-      <c r="S23" s="2"/>
+        <v>1932993.8565</v>
+      </c>
       <c r="T23">
-        <v>65659.95</v>
+        <v>182026.51</v>
       </c>
       <c r="U23">
-        <v>65659.95</v>
+        <v>232026.51</v>
       </c>
       <c r="V23">
-        <v>65659.95</v>
+        <v>273039.76500000001</v>
       </c>
       <c r="W23">
-        <v>65659.95</v>
+        <v>273039.76500000001</v>
       </c>
       <c r="X23">
-        <v>65659.95</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>273039.76500000001</v>
+      </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -4911,66 +4645,62 @@
         <v>179454.27239999999</v>
       </c>
       <c r="C24">
-        <v>179454.27239999999</v>
+        <v>229454.27239999999</v>
       </c>
       <c r="D24">
-        <v>179454.27239999999</v>
+        <v>269181.40860000002</v>
       </c>
       <c r="E24">
-        <v>179454.27239999999</v>
+        <v>269181.40860000002</v>
       </c>
       <c r="F24">
-        <v>179454.27239999999</v>
-      </c>
-      <c r="G24" s="2"/>
+        <v>269181.40860000002</v>
+      </c>
       <c r="H24">
         <v>964055.63519999932</v>
       </c>
       <c r="I24">
-        <v>964055.63519999932</v>
-      </c>
-      <c r="J24">
-        <v>964055.63519999932</v>
-      </c>
-      <c r="K24">
-        <v>964055.63519999932</v>
-      </c>
-      <c r="L24">
-        <v>964055.63519999932</v>
-      </c>
-      <c r="M24" s="2"/>
+        <v>1014055.6352</v>
+      </c>
+      <c r="J24" s="4">
+        <v>1446083.4528000001</v>
+      </c>
+      <c r="K24" s="4">
+        <v>1446083.4528000001</v>
+      </c>
+      <c r="L24" s="4">
+        <v>1446083.4528000001</v>
+      </c>
       <c r="N24">
         <v>1288789.5264390404</v>
       </c>
       <c r="O24">
-        <v>1288789.5264390404</v>
+        <v>1338789.5260000001</v>
       </c>
       <c r="P24">
-        <v>1288789.5264390404</v>
+        <v>1933184.2890000001</v>
       </c>
       <c r="Q24">
-        <v>1288789.5264390404</v>
+        <v>1933184.2890000001</v>
       </c>
       <c r="R24">
-        <v>1288789.5264390404</v>
-      </c>
-      <c r="S24" s="2"/>
+        <v>1933184.2890000001</v>
+      </c>
       <c r="T24">
-        <v>64674.05</v>
+        <v>178332.87</v>
       </c>
       <c r="U24">
-        <v>64674.05</v>
+        <v>228332.87</v>
       </c>
       <c r="V24">
-        <v>64674.05</v>
+        <v>267499.30499999999</v>
       </c>
       <c r="W24">
-        <v>64674.05</v>
+        <v>267499.30499999999</v>
       </c>
       <c r="X24">
-        <v>64674.05</v>
-      </c>
-      <c r="Y24" s="2"/>
+        <v>267499.30499999999</v>
+      </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -4980,66 +4710,62 @@
         <v>176762.4583</v>
       </c>
       <c r="C25">
-        <v>176762.4583</v>
+        <v>226762.4583</v>
       </c>
       <c r="D25">
-        <v>176762.4583</v>
+        <v>265143.68745000003</v>
       </c>
       <c r="E25">
-        <v>176762.4583</v>
+        <v>265143.68745000003</v>
       </c>
       <c r="F25">
-        <v>176762.4583</v>
-      </c>
-      <c r="G25" s="2"/>
+        <v>265143.68745000003</v>
+      </c>
       <c r="H25">
         <v>962142.82639999932</v>
       </c>
       <c r="I25">
-        <v>962142.82639999932</v>
-      </c>
-      <c r="J25">
-        <v>962142.82639999932</v>
-      </c>
-      <c r="K25">
-        <v>962142.82639999932</v>
-      </c>
-      <c r="L25">
-        <v>962142.82639999932</v>
-      </c>
-      <c r="M25" s="2"/>
+        <v>1012142.8264</v>
+      </c>
+      <c r="J25" s="4">
+        <v>1443214.2396</v>
+      </c>
+      <c r="K25" s="4">
+        <v>1443214.2396</v>
+      </c>
+      <c r="L25" s="4">
+        <v>1443214.2396</v>
+      </c>
       <c r="N25">
         <v>1288916.4815234803</v>
       </c>
       <c r="O25">
-        <v>1288916.4815234803</v>
+        <v>1338916.4820000001</v>
       </c>
       <c r="P25">
-        <v>1288916.4815234803</v>
+        <v>1933374.723</v>
       </c>
       <c r="Q25">
-        <v>1288916.4815234803</v>
+        <v>1933374.723</v>
       </c>
       <c r="R25">
-        <v>1288916.4815234803</v>
-      </c>
-      <c r="S25" s="2"/>
+        <v>1933374.723</v>
+      </c>
       <c r="T25">
-        <v>63702.94</v>
+        <v>174720.11</v>
       </c>
       <c r="U25">
-        <v>63702.94</v>
+        <v>224720.11</v>
       </c>
       <c r="V25">
-        <v>63702.94</v>
+        <v>262080.16500000001</v>
       </c>
       <c r="W25">
-        <v>63702.94</v>
+        <v>262080.16500000001</v>
       </c>
       <c r="X25">
-        <v>63702.94</v>
-      </c>
-      <c r="Y25" s="2"/>
+        <v>262080.16500000001</v>
+      </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -5049,66 +4775,62 @@
         <v>174111.0214</v>
       </c>
       <c r="C26">
-        <v>174111.0214</v>
+        <v>224111.0214</v>
       </c>
       <c r="D26">
-        <v>174111.0214</v>
+        <v>261166.53210000001</v>
       </c>
       <c r="E26">
-        <v>174111.0214</v>
+        <v>261166.53210000001</v>
       </c>
       <c r="F26">
-        <v>174111.0214</v>
-      </c>
-      <c r="G26" s="2"/>
+        <v>261166.53210000001</v>
+      </c>
       <c r="H26">
         <v>960230.01759999921</v>
       </c>
       <c r="I26">
-        <v>960230.01759999921</v>
-      </c>
-      <c r="J26">
-        <v>960230.01759999921</v>
-      </c>
-      <c r="K26">
-        <v>960230.01759999921</v>
-      </c>
-      <c r="L26">
-        <v>960230.01759999921</v>
-      </c>
-      <c r="M26" s="2"/>
+        <v>1010230.0176</v>
+      </c>
+      <c r="J26" s="4">
+        <v>1440345.0264000001</v>
+      </c>
+      <c r="K26" s="4">
+        <v>1440345.0264000001</v>
+      </c>
+      <c r="L26" s="4">
+        <v>1440345.0264000001</v>
+      </c>
       <c r="N26">
         <v>1289043.4366079206</v>
       </c>
       <c r="O26">
-        <v>1289043.4366079206</v>
+        <v>1339043.4369999999</v>
       </c>
       <c r="P26">
-        <v>1289043.4366079206</v>
+        <v>1933565.1555000001</v>
       </c>
       <c r="Q26">
-        <v>1289043.4366079206</v>
+        <v>1933565.1555000001</v>
       </c>
       <c r="R26">
-        <v>1289043.4366079206</v>
-      </c>
-      <c r="S26" s="2"/>
+        <v>1933565.1555000001</v>
+      </c>
       <c r="T26">
-        <v>62746.400000000001</v>
+        <v>171187.17</v>
       </c>
       <c r="U26">
-        <v>62746.400000000001</v>
+        <v>221187.17</v>
       </c>
       <c r="V26">
-        <v>62746.400000000001</v>
+        <v>256780.755</v>
       </c>
       <c r="W26">
-        <v>62746.400000000001</v>
+        <v>256780.755</v>
       </c>
       <c r="X26">
-        <v>62746.400000000001</v>
-      </c>
-      <c r="Y26" s="2"/>
+        <v>256780.755</v>
+      </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27">
@@ -5118,73 +4840,73 @@
         <v>171499.3561</v>
       </c>
       <c r="C27">
-        <v>171499.3561</v>
+        <v>221499.3561</v>
       </c>
       <c r="D27">
-        <v>171499.3561</v>
+        <v>257249.03414999999</v>
       </c>
       <c r="E27">
-        <v>171499.3561</v>
+        <v>257249.03414999999</v>
       </c>
       <c r="F27">
-        <v>171499.3561</v>
+        <v>257249.03414999999</v>
       </c>
       <c r="G27">
-        <v>171499.3561</v>
+        <v>257249.03414999999</v>
       </c>
       <c r="H27">
         <v>958317.20879999921</v>
       </c>
       <c r="I27">
-        <v>958317.20879999921</v>
-      </c>
-      <c r="J27">
-        <v>958317.20879999921</v>
-      </c>
-      <c r="K27">
-        <v>958317.20879999921</v>
-      </c>
-      <c r="L27">
-        <v>958317.20879999921</v>
-      </c>
-      <c r="M27">
-        <v>958317.20879999921</v>
+        <v>1008317.2088</v>
+      </c>
+      <c r="J27" s="4">
+        <v>1437475.8132</v>
+      </c>
+      <c r="K27" s="4">
+        <v>1437475.8132</v>
+      </c>
+      <c r="L27" s="4">
+        <v>1437475.8132</v>
+      </c>
+      <c r="M27" s="4">
+        <v>1437475.8132</v>
       </c>
       <c r="N27">
         <v>1289170.3916923604</v>
       </c>
       <c r="O27">
-        <v>1289170.3916923604</v>
+        <v>1339170.392</v>
       </c>
       <c r="P27">
-        <v>1289170.3916923604</v>
+        <v>1933755.588</v>
       </c>
       <c r="Q27">
-        <v>1289170.3916923604</v>
+        <v>1933755.588</v>
       </c>
       <c r="R27">
-        <v>1289170.3916923604</v>
+        <v>1933755.588</v>
       </c>
       <c r="S27">
-        <v>1289170.3916923604</v>
+        <v>1933755.588</v>
       </c>
       <c r="T27">
-        <v>61804.2</v>
+        <v>167732.98000000001</v>
       </c>
       <c r="U27">
-        <v>61804.2</v>
+        <v>217732.98</v>
       </c>
       <c r="V27">
-        <v>61804.2</v>
+        <v>251599.47</v>
       </c>
       <c r="W27">
-        <v>61804.2</v>
+        <v>251599.47</v>
       </c>
       <c r="X27">
-        <v>61804.2</v>
+        <v>251599.47</v>
       </c>
       <c r="Y27">
-        <v>61804.2</v>
+        <v>251599.47</v>
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.3">
@@ -5195,73 +4917,73 @@
         <v>168926.8658</v>
       </c>
       <c r="C28">
-        <v>168926.8658</v>
+        <v>218926.8658</v>
       </c>
       <c r="D28">
-        <v>168926.8658</v>
+        <v>253390.29870000001</v>
       </c>
       <c r="E28">
-        <v>168926.8658</v>
+        <v>253390.29870000001</v>
       </c>
       <c r="F28">
-        <v>168926.8658</v>
+        <v>253390.29870000001</v>
       </c>
       <c r="G28">
-        <v>168926.8658</v>
+        <v>253390.29870000001</v>
       </c>
       <c r="H28">
         <v>956404.40000000026</v>
       </c>
       <c r="I28">
-        <v>956404.40000000026</v>
-      </c>
-      <c r="J28">
-        <v>956404.40000000026</v>
-      </c>
-      <c r="K28">
-        <v>956404.40000000026</v>
-      </c>
-      <c r="L28">
-        <v>956404.40000000026</v>
-      </c>
-      <c r="M28">
-        <v>956404.40000000026</v>
+        <v>1006404.4</v>
+      </c>
+      <c r="J28" s="4">
+        <v>1434606.6</v>
+      </c>
+      <c r="K28" s="4">
+        <v>1434606.6</v>
+      </c>
+      <c r="L28" s="4">
+        <v>1434606.6</v>
+      </c>
+      <c r="M28" s="4">
+        <v>1434606.6</v>
       </c>
       <c r="N28">
         <v>1289297.3467768</v>
       </c>
       <c r="O28">
-        <v>1289297.3467768</v>
+        <v>1339297.3470000001</v>
       </c>
       <c r="P28">
-        <v>1289297.3467768</v>
+        <v>1933946.0205000001</v>
       </c>
       <c r="Q28">
-        <v>1289297.3467768</v>
+        <v>1933946.0205000001</v>
       </c>
       <c r="R28">
-        <v>1289297.3467768</v>
+        <v>1933946.0205000001</v>
       </c>
       <c r="S28">
-        <v>1289297.3467768</v>
+        <v>1933946.0205000001</v>
       </c>
       <c r="T28">
-        <v>60876.14</v>
+        <v>164356.51999999999</v>
       </c>
       <c r="U28">
-        <v>60876.14</v>
+        <v>214356.52</v>
       </c>
       <c r="V28">
-        <v>60876.14</v>
+        <v>246534.78</v>
       </c>
       <c r="W28">
-        <v>60876.14</v>
+        <v>246534.78</v>
       </c>
       <c r="X28">
-        <v>60876.14</v>
+        <v>246534.78</v>
       </c>
       <c r="Y28">
-        <v>60876.14</v>
+        <v>246534.78</v>
       </c>
     </row>
   </sheetData>
@@ -5278,79 +5000,79 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
     <row r="1" spans="1:25" x14ac:dyDescent="0.3">
-      <c r="A1" t="s">
+      <c r="A1" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
+      <c r="B1" s="3" t="s">
         <v>44</v>
       </c>
-      <c r="C1" t="s">
+      <c r="C1" s="3" t="s">
         <v>45</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="3" t="s">
         <v>47</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="3" t="s">
         <v>48</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="3" t="s">
         <v>49</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="3" t="s">
         <v>51</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="3" t="s">
         <v>52</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="3" t="s">
         <v>53</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="3" t="s">
         <v>54</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="3" t="s">
         <v>55</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="3" t="s">
         <v>56</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="3" t="s">
         <v>57</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="3" t="s">
         <v>58</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="3" t="s">
         <v>59</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="3" t="s">
         <v>60</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="3" t="s">
         <v>61</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="3" t="s">
         <v>62</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="3" t="s">
         <v>63</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="3" t="s">
         <v>64</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="3" t="s">
         <v>65</v>
       </c>
-      <c r="X1" t="s">
+      <c r="X1" s="3" t="s">
         <v>66</v>
       </c>
-      <c r="Y1" t="s">
+      <c r="Y1" s="3" t="s">
         <v>67</v>
       </c>
     </row>
@@ -5361,35 +5083,15 @@
       <c r="B2">
         <v>303600</v>
       </c>
-      <c r="C2" s="2"/>
-      <c r="D2" s="2"/>
-      <c r="E2" s="2"/>
-      <c r="F2" s="2"/>
-      <c r="G2" s="2"/>
       <c r="H2">
         <v>1673707.7</v>
       </c>
-      <c r="I2" s="2"/>
-      <c r="J2" s="2"/>
-      <c r="K2" s="2"/>
-      <c r="L2" s="2"/>
-      <c r="M2" s="2"/>
       <c r="N2">
         <v>2337972.5216000001</v>
       </c>
-      <c r="O2" s="2"/>
-      <c r="P2" s="2"/>
-      <c r="Q2" s="2"/>
-      <c r="R2" s="2"/>
-      <c r="S2" s="2"/>
-      <c r="T2" s="3">
-        <v>129380</v>
-      </c>
-      <c r="U2" s="2"/>
-      <c r="V2" s="2"/>
-      <c r="W2" s="2"/>
-      <c r="X2" s="2"/>
-      <c r="Y2" s="2"/>
+      <c r="T2">
+        <v>527469.86</v>
+      </c>
     </row>
     <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3">
@@ -5398,35 +5100,15 @@
       <c r="B3">
         <v>299045.40000000002</v>
       </c>
-      <c r="C3" s="2"/>
-      <c r="D3" s="2"/>
-      <c r="E3" s="2"/>
-      <c r="F3" s="2"/>
-      <c r="G3" s="2"/>
       <c r="H3">
         <v>1660955.6413333334</v>
       </c>
-      <c r="I3" s="2"/>
-      <c r="J3" s="2"/>
-      <c r="K3" s="2"/>
-      <c r="L3" s="2"/>
-      <c r="M3" s="2"/>
       <c r="N3">
         <v>2318026.381866667</v>
       </c>
-      <c r="O3" s="2"/>
-      <c r="P3" s="2"/>
-      <c r="Q3" s="2"/>
-      <c r="R3" s="2"/>
-      <c r="S3" s="2"/>
-      <c r="T3" s="3">
-        <v>127438.3</v>
-      </c>
-      <c r="U3" s="2"/>
-      <c r="V3" s="2"/>
-      <c r="W3" s="2"/>
-      <c r="X3" s="2"/>
-      <c r="Y3" s="2"/>
+      <c r="T3">
+        <v>516785.56</v>
+      </c>
     </row>
     <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4">
@@ -5435,35 +5117,15 @@
       <c r="B4">
         <v>294559.71899999998</v>
       </c>
-      <c r="C4" s="2"/>
-      <c r="D4" s="2"/>
-      <c r="E4" s="2"/>
-      <c r="F4" s="2"/>
-      <c r="G4" s="2"/>
       <c r="H4">
         <v>1648203.5826666667</v>
       </c>
-      <c r="I4" s="2"/>
-      <c r="J4" s="2"/>
-      <c r="K4" s="2"/>
-      <c r="L4" s="2"/>
-      <c r="M4" s="2"/>
       <c r="N4">
         <v>2298080.2421333333</v>
       </c>
-      <c r="O4" s="2"/>
-      <c r="P4" s="2"/>
-      <c r="Q4" s="2"/>
-      <c r="R4" s="2"/>
-      <c r="S4" s="2"/>
-      <c r="T4" s="3">
-        <v>125526.73</v>
-      </c>
-      <c r="U4" s="2"/>
-      <c r="V4" s="2"/>
-      <c r="W4" s="2"/>
-      <c r="X4" s="2"/>
-      <c r="Y4" s="2"/>
+      <c r="T4">
+        <v>506302.5</v>
+      </c>
     </row>
     <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5">
@@ -5472,35 +5134,15 @@
       <c r="B5">
         <v>290141.32319999998</v>
       </c>
-      <c r="C5" s="2"/>
-      <c r="D5" s="2"/>
-      <c r="E5" s="2"/>
-      <c r="F5" s="2"/>
-      <c r="G5" s="2"/>
       <c r="H5">
         <v>1635451.524</v>
       </c>
-      <c r="I5" s="2"/>
-      <c r="J5" s="2"/>
-      <c r="K5" s="2"/>
-      <c r="L5" s="2"/>
-      <c r="M5" s="2"/>
       <c r="N5">
         <v>2278134.1023999997</v>
       </c>
-      <c r="O5" s="2"/>
-      <c r="P5" s="2"/>
-      <c r="Q5" s="2"/>
-      <c r="R5" s="2"/>
-      <c r="S5" s="2"/>
-      <c r="T5" s="3">
-        <v>123644.83</v>
-      </c>
-      <c r="U5" s="2"/>
-      <c r="V5" s="2"/>
-      <c r="W5" s="2"/>
-      <c r="X5" s="2"/>
-      <c r="Y5" s="2"/>
+      <c r="T5">
+        <v>496017.89</v>
+      </c>
     </row>
     <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6">
@@ -5509,35 +5151,15 @@
       <c r="B6">
         <v>285788.2034</v>
       </c>
-      <c r="C6" s="2"/>
-      <c r="D6" s="2"/>
-      <c r="E6" s="2"/>
-      <c r="F6" s="2"/>
-      <c r="G6" s="2"/>
       <c r="H6">
         <v>1622699.4653333335</v>
       </c>
-      <c r="I6" s="2"/>
-      <c r="J6" s="2"/>
-      <c r="K6" s="2"/>
-      <c r="L6" s="2"/>
-      <c r="M6" s="2"/>
       <c r="N6">
         <v>2258187.9626666661</v>
       </c>
-      <c r="O6" s="2"/>
-      <c r="P6" s="2"/>
-      <c r="Q6" s="2"/>
-      <c r="R6" s="2"/>
-      <c r="S6" s="2"/>
-      <c r="T6" s="3">
-        <v>121792.16</v>
-      </c>
-      <c r="U6" s="2"/>
-      <c r="V6" s="2"/>
-      <c r="W6" s="2"/>
-      <c r="X6" s="2"/>
-      <c r="Y6" s="2"/>
+      <c r="T6">
+        <v>485929.01</v>
+      </c>
     </row>
     <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7">
@@ -5549,40 +5171,24 @@
       <c r="C7">
         <v>281498.4804</v>
       </c>
-      <c r="D7" s="2"/>
-      <c r="E7" s="2"/>
-      <c r="F7" s="2"/>
-      <c r="G7" s="2"/>
       <c r="H7">
         <v>1609947.4066666667</v>
       </c>
       <c r="I7">
         <v>1609947.4066666667</v>
       </c>
-      <c r="J7" s="2"/>
-      <c r="K7" s="2"/>
-      <c r="L7" s="2"/>
-      <c r="M7" s="2"/>
       <c r="N7">
         <v>2238241.8229333302</v>
       </c>
       <c r="O7">
         <v>2238241.8229333302</v>
       </c>
-      <c r="P7" s="2"/>
-      <c r="Q7" s="2"/>
-      <c r="R7" s="2"/>
-      <c r="S7" s="2"/>
-      <c r="T7" s="3">
-        <v>119968.28</v>
-      </c>
-      <c r="U7" s="3">
-        <v>119968.28</v>
-      </c>
-      <c r="V7" s="2"/>
-      <c r="W7" s="2"/>
-      <c r="X7" s="2"/>
-      <c r="Y7" s="2"/>
+      <c r="T7">
+        <v>476033.18</v>
+      </c>
+      <c r="U7">
+        <v>476033.18</v>
+      </c>
     </row>
     <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8">
@@ -5592,42 +5198,26 @@
         <v>277270.34419999999</v>
       </c>
       <c r="C8">
-        <v>277270.34419999999</v>
-      </c>
-      <c r="D8" s="2"/>
-      <c r="E8" s="2"/>
-      <c r="F8" s="2"/>
-      <c r="G8" s="2"/>
+        <v>207952.75815000001</v>
+      </c>
       <c r="H8">
         <v>1597195.3480000002</v>
       </c>
       <c r="I8">
-        <v>1597195.3480000002</v>
-      </c>
-      <c r="J8" s="2"/>
-      <c r="K8" s="2"/>
-      <c r="L8" s="2"/>
-      <c r="M8" s="2"/>
+        <v>1197896.5109999999</v>
+      </c>
       <c r="N8">
         <v>2218295.6831999999</v>
       </c>
       <c r="O8">
-        <v>2218295.6831999999</v>
-      </c>
-      <c r="P8" s="2"/>
-      <c r="Q8" s="2"/>
-      <c r="R8" s="2"/>
-      <c r="S8" s="2"/>
-      <c r="T8" s="3">
-        <v>118172.75</v>
-      </c>
-      <c r="U8" s="3">
-        <v>118172.75</v>
-      </c>
-      <c r="V8" s="2"/>
-      <c r="W8" s="2"/>
-      <c r="X8" s="2"/>
-      <c r="Y8" s="2"/>
+        <v>1663721.7622499999</v>
+      </c>
+      <c r="T8">
+        <v>466327.8</v>
+      </c>
+      <c r="U8">
+        <v>349745.85</v>
+      </c>
     </row>
     <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9">
@@ -5637,42 +5227,26 @@
         <v>273102.28909999999</v>
       </c>
       <c r="C9">
-        <v>273102.28909999999</v>
-      </c>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
-      <c r="G9" s="2"/>
+        <v>204826.71682500001</v>
+      </c>
       <c r="H9">
         <v>1594326.1348000003</v>
       </c>
       <c r="I9">
-        <v>1594326.1348000003</v>
-      </c>
-      <c r="J9" s="2"/>
-      <c r="K9" s="2"/>
-      <c r="L9" s="2"/>
-      <c r="M9" s="2"/>
+        <v>1195744.6012500001</v>
+      </c>
       <c r="N9">
         <v>2205259.4561600001</v>
       </c>
       <c r="O9">
-        <v>2205259.4561600001</v>
-      </c>
-      <c r="P9" s="2"/>
-      <c r="Q9" s="2"/>
-      <c r="R9" s="2"/>
-      <c r="S9" s="2"/>
-      <c r="T9" s="3">
-        <v>116405.16</v>
-      </c>
-      <c r="U9" s="3">
-        <v>116405.16</v>
-      </c>
-      <c r="V9" s="2"/>
-      <c r="W9" s="2"/>
-      <c r="X9" s="2"/>
-      <c r="Y9" s="2"/>
+        <v>1653944.5919999999</v>
+      </c>
+      <c r="T9">
+        <v>456810.3</v>
+      </c>
+      <c r="U9">
+        <v>342607.72499999998</v>
+      </c>
     </row>
     <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10">
@@ -5682,42 +5256,26 @@
         <v>268993.2548</v>
       </c>
       <c r="C10">
-        <v>268993.2548</v>
-      </c>
-      <c r="D10" s="2"/>
-      <c r="E10" s="2"/>
-      <c r="F10" s="2"/>
-      <c r="G10" s="2"/>
+        <v>201744.9411</v>
+      </c>
       <c r="H10">
         <v>1591456.9216000002</v>
       </c>
       <c r="I10">
-        <v>1591456.9216000002</v>
-      </c>
-      <c r="J10" s="2"/>
-      <c r="K10" s="2"/>
-      <c r="L10" s="2"/>
-      <c r="M10" s="2"/>
+        <v>1193592.6915</v>
+      </c>
       <c r="N10">
         <v>2192223.2291199998</v>
       </c>
       <c r="O10">
-        <v>2192223.2291199998</v>
-      </c>
-      <c r="P10" s="2"/>
-      <c r="Q10" s="2"/>
-      <c r="R10" s="2"/>
-      <c r="S10" s="2"/>
-      <c r="T10" s="3">
-        <v>114665.09</v>
-      </c>
-      <c r="U10" s="3">
-        <v>114665.09</v>
-      </c>
-      <c r="V10" s="2"/>
-      <c r="W10" s="2"/>
-      <c r="X10" s="2"/>
-      <c r="Y10" s="2"/>
+        <v>1644167.42175</v>
+      </c>
+      <c r="T10">
+        <v>447478.16</v>
+      </c>
+      <c r="U10">
+        <v>335608.62</v>
+      </c>
     </row>
     <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11">
@@ -5727,42 +5285,26 @@
         <v>264942.41499999998</v>
       </c>
       <c r="C11">
-        <v>264942.41499999998</v>
-      </c>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
-      <c r="G11" s="2"/>
+        <v>198706.81125</v>
+      </c>
       <c r="H11">
         <v>1588587.7084000004</v>
       </c>
       <c r="I11">
-        <v>1588587.7084000004</v>
-      </c>
-      <c r="J11" s="2"/>
-      <c r="K11" s="2"/>
-      <c r="L11" s="2"/>
-      <c r="M11" s="2"/>
+        <v>1191440.781</v>
+      </c>
       <c r="N11">
         <v>2179187.0020799995</v>
       </c>
       <c r="O11">
-        <v>2179187.0020799995</v>
-      </c>
-      <c r="P11" s="2"/>
-      <c r="Q11" s="2"/>
-      <c r="R11" s="2"/>
-      <c r="S11" s="2"/>
-      <c r="T11" s="3">
-        <v>112952.12</v>
-      </c>
-      <c r="U11" s="3">
-        <v>112952.12</v>
-      </c>
-      <c r="V11" s="2"/>
-      <c r="W11" s="2"/>
-      <c r="X11" s="2"/>
-      <c r="Y11" s="2"/>
+        <v>1634390.2515</v>
+      </c>
+      <c r="T11">
+        <v>438328.91</v>
+      </c>
+      <c r="U11">
+        <v>328746.6825</v>
+      </c>
     </row>
     <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12">
@@ -5772,50 +5314,38 @@
         <v>260948.7948</v>
       </c>
       <c r="C12">
-        <v>260948.7948</v>
+        <v>195711.5961</v>
       </c>
       <c r="D12">
-        <v>260948.7948</v>
-      </c>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
-      <c r="G12" s="2"/>
+        <v>195711.5961</v>
+      </c>
       <c r="H12">
         <v>1585718.4952000002</v>
       </c>
       <c r="I12">
-        <v>1585718.4952000002</v>
+        <v>1189288.87075</v>
       </c>
       <c r="J12">
-        <v>1585718.4952000002</v>
-      </c>
-      <c r="K12" s="2"/>
-      <c r="L12" s="2"/>
-      <c r="M12" s="2"/>
+        <v>1189288.87075</v>
+      </c>
       <c r="N12">
         <v>2166150.7750399997</v>
       </c>
       <c r="O12">
-        <v>2166150.7750399997</v>
+        <v>1624613.08125</v>
       </c>
       <c r="P12">
-        <v>2166150.7750399997</v>
-      </c>
-      <c r="Q12" s="2"/>
-      <c r="R12" s="2"/>
-      <c r="S12" s="2"/>
-      <c r="T12" s="3">
-        <v>111265.84</v>
-      </c>
-      <c r="U12" s="3">
-        <v>111265.84</v>
-      </c>
-      <c r="V12" s="3">
-        <v>111265.84</v>
-      </c>
-      <c r="W12" s="2"/>
-      <c r="X12" s="2"/>
-      <c r="Y12" s="2"/>
+        <v>1624613.08125</v>
+      </c>
+      <c r="T12">
+        <v>429360.14</v>
+      </c>
+      <c r="U12">
+        <v>322020.10499999998</v>
+      </c>
+      <c r="V12">
+        <v>322020.10499999998</v>
+      </c>
     </row>
     <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13">
@@ -5825,50 +5355,38 @@
         <v>257011.4613</v>
       </c>
       <c r="C13">
-        <v>257011.4613</v>
+        <v>192758.595975</v>
       </c>
       <c r="D13">
-        <v>257011.4613</v>
-      </c>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
-      <c r="G13" s="2"/>
+        <v>289137.89399999997</v>
+      </c>
       <c r="H13">
         <v>1582849.2820000004</v>
       </c>
       <c r="I13">
-        <v>1582849.2820000004</v>
+        <v>1187136.9605</v>
       </c>
       <c r="J13">
-        <v>1582849.2820000004</v>
-      </c>
-      <c r="K13" s="2"/>
-      <c r="L13" s="2"/>
-      <c r="M13" s="2"/>
+        <v>1780705.4415</v>
+      </c>
       <c r="N13">
         <v>2153114.5479999995</v>
       </c>
       <c r="O13">
-        <v>2153114.5479999995</v>
+        <v>1614835.9110000001</v>
       </c>
       <c r="P13">
-        <v>2153114.5479999995</v>
-      </c>
-      <c r="Q13" s="2"/>
-      <c r="R13" s="2"/>
-      <c r="S13" s="2"/>
-      <c r="T13" s="3">
-        <v>109605.86</v>
-      </c>
-      <c r="U13" s="3">
-        <v>109605.86</v>
-      </c>
-      <c r="V13" s="3">
-        <v>109605.86</v>
-      </c>
-      <c r="W13" s="2"/>
-      <c r="X13" s="2"/>
-      <c r="Y13" s="2"/>
+        <v>2422253.8665</v>
+      </c>
+      <c r="T13">
+        <v>420569.49</v>
+      </c>
+      <c r="U13">
+        <v>473140.67625000002</v>
+      </c>
+      <c r="V13">
+        <v>709711.01445000002</v>
+      </c>
     </row>
     <row r="14" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A14">
@@ -5878,50 +5396,38 @@
         <v>253129.39139999999</v>
       </c>
       <c r="C14">
-        <v>253129.39139999999</v>
+        <v>189847.04355</v>
       </c>
       <c r="D14">
-        <v>253129.39139999999</v>
-      </c>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
-      <c r="G14" s="2"/>
+        <v>284770.56540000002</v>
+      </c>
       <c r="H14">
         <v>1579980.0688000005</v>
       </c>
       <c r="I14">
-        <v>1579980.0688000005</v>
+        <v>1184985.0507499999</v>
       </c>
       <c r="J14">
-        <v>1579980.0688000005</v>
-      </c>
-      <c r="K14" s="2"/>
-      <c r="L14" s="2"/>
-      <c r="M14" s="2"/>
+        <v>1777477.5765</v>
+      </c>
       <c r="N14">
         <v>2140078.3209599997</v>
       </c>
       <c r="O14">
-        <v>2140078.3209599997</v>
+        <v>1605058.7407500001</v>
       </c>
       <c r="P14">
-        <v>2140078.3209599997</v>
-      </c>
-      <c r="Q14" s="2"/>
-      <c r="R14" s="2"/>
-      <c r="S14" s="2"/>
-      <c r="T14" s="3">
-        <v>107971.77</v>
-      </c>
-      <c r="U14" s="3">
-        <v>107971.77</v>
-      </c>
-      <c r="V14" s="3">
-        <v>107971.77</v>
-      </c>
-      <c r="W14" s="2"/>
-      <c r="X14" s="2"/>
-      <c r="Y14" s="2"/>
+        <v>2407588.1115000001</v>
+      </c>
+      <c r="T14">
+        <v>411954.65</v>
+      </c>
+      <c r="U14">
+        <v>463450.48125000001</v>
+      </c>
+      <c r="V14">
+        <v>695175.72195000004</v>
+      </c>
     </row>
     <row r="15" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A15">
@@ -5931,50 +5437,38 @@
         <v>249301.63759999999</v>
       </c>
       <c r="C15">
-        <v>249301.63759999999</v>
+        <v>186976.22820000001</v>
       </c>
       <c r="D15">
-        <v>249301.63759999999</v>
-      </c>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
-      <c r="G15" s="2"/>
+        <v>280464.34230000002</v>
+      </c>
       <c r="H15">
         <v>1577110.8556000004</v>
       </c>
       <c r="I15">
-        <v>1577110.8556000004</v>
+        <v>1182833.14075</v>
       </c>
       <c r="J15">
-        <v>1577110.8556000004</v>
-      </c>
-      <c r="K15" s="2"/>
-      <c r="L15" s="2"/>
-      <c r="M15" s="2"/>
+        <v>1774250.7115</v>
+      </c>
       <c r="N15">
         <v>2127042.0939199994</v>
       </c>
       <c r="O15">
-        <v>2127042.0939199994</v>
+        <v>1595281.5704999999</v>
       </c>
       <c r="P15">
-        <v>2127042.0939199994</v>
-      </c>
-      <c r="Q15" s="2"/>
-      <c r="R15" s="2"/>
-      <c r="S15" s="2"/>
+        <v>2392922.3565000002</v>
+      </c>
       <c r="T15">
-        <v>106363.2</v>
+        <v>403513.36</v>
       </c>
       <c r="U15">
-        <v>106363.2</v>
+        <v>453952.53</v>
       </c>
       <c r="V15">
-        <v>106363.2</v>
-      </c>
-      <c r="W15" s="2"/>
-      <c r="X15" s="2"/>
-      <c r="Y15" s="2"/>
+        <v>680928.79500000004</v>
+      </c>
     </row>
     <row r="16" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A16">
@@ -5984,50 +5478,38 @@
         <v>245527.30809999999</v>
       </c>
       <c r="C16">
-        <v>245527.30809999999</v>
+        <v>184145.48107499999</v>
       </c>
       <c r="D16">
-        <v>245527.30809999999</v>
-      </c>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
-      <c r="G16" s="2"/>
+        <v>276218.22169999999</v>
+      </c>
       <c r="H16">
         <v>1574241.6424000005</v>
       </c>
       <c r="I16">
-        <v>1574241.6424000005</v>
+        <v>1180681.2315</v>
       </c>
       <c r="J16">
-        <v>1574241.6424000005</v>
-      </c>
-      <c r="K16" s="2"/>
-      <c r="L16" s="2"/>
-      <c r="M16" s="2"/>
+        <v>1771023.848</v>
+      </c>
       <c r="N16">
         <v>2114005.8668799992</v>
       </c>
       <c r="O16">
-        <v>2114005.8668799992</v>
+        <v>1585504.4002499999</v>
       </c>
       <c r="P16">
-        <v>2114005.8668799992</v>
-      </c>
-      <c r="Q16" s="2"/>
-      <c r="R16" s="2"/>
-      <c r="S16" s="2"/>
+        <v>2378256.6</v>
+      </c>
       <c r="T16">
-        <v>104779.75</v>
+        <v>395243.39</v>
       </c>
       <c r="U16">
-        <v>104779.75</v>
+        <v>444648.81374999997</v>
       </c>
       <c r="V16">
-        <v>104779.75</v>
-      </c>
-      <c r="W16" s="2"/>
-      <c r="X16" s="2"/>
-      <c r="Y16" s="2"/>
+        <v>666973.22069999995</v>
+      </c>
     </row>
     <row r="17" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A17">
@@ -6037,58 +5519,50 @@
         <v>241805.39859999999</v>
       </c>
       <c r="C17">
-        <v>241805.39859999999</v>
+        <v>181354.04934999999</v>
       </c>
       <c r="D17">
-        <v>241805.39859999999</v>
+        <v>272031.07410000003</v>
       </c>
       <c r="E17">
-        <v>241805.39859999999</v>
-      </c>
-      <c r="F17" s="2"/>
-      <c r="G17" s="2"/>
+        <v>272031.07410000003</v>
+      </c>
       <c r="H17">
         <v>1571372.4292000004</v>
       </c>
       <c r="I17">
-        <v>1571372.4292000004</v>
+        <v>1178529.3217499999</v>
       </c>
       <c r="J17">
-        <v>1571372.4292000004</v>
+        <v>1767796.983</v>
       </c>
       <c r="K17">
-        <v>1571372.4292000004</v>
-      </c>
-      <c r="L17" s="2"/>
-      <c r="M17" s="2"/>
+        <v>1767796.983</v>
+      </c>
       <c r="N17">
         <v>2100969.6398399994</v>
       </c>
       <c r="O17">
-        <v>2100969.6398399994</v>
+        <v>1575727.23</v>
       </c>
       <c r="P17">
-        <v>2100969.6398399994</v>
+        <v>2363590.8450000002</v>
       </c>
       <c r="Q17">
-        <v>2100969.6398399994</v>
-      </c>
-      <c r="R17" s="2"/>
-      <c r="S17" s="2"/>
+        <v>2363590.8450000002</v>
+      </c>
       <c r="T17">
-        <v>103221.06</v>
+        <v>387142.59</v>
       </c>
       <c r="U17">
-        <v>103221.06</v>
+        <v>435535.41375000001</v>
       </c>
       <c r="V17">
-        <v>103221.06</v>
+        <v>653303.12069999997</v>
       </c>
       <c r="W17">
-        <v>103221.06</v>
-      </c>
-      <c r="X17" s="2"/>
-      <c r="Y17" s="2"/>
+        <v>653303.12069999997</v>
+      </c>
     </row>
     <row r="18" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A18">
@@ -6098,58 +5572,50 @@
         <v>238134.9901</v>
       </c>
       <c r="C18">
-        <v>238134.9901</v>
+        <v>178601.24257500001</v>
       </c>
       <c r="D18">
-        <v>238134.9901</v>
+        <v>267901.864</v>
       </c>
       <c r="E18">
-        <v>238134.9901</v>
-      </c>
-      <c r="F18" s="2"/>
-      <c r="G18" s="2"/>
+        <v>267901.864</v>
+      </c>
       <c r="H18">
         <v>1568503.2160000005</v>
       </c>
       <c r="I18">
-        <v>1568503.2160000005</v>
+        <v>1176377.412</v>
       </c>
       <c r="J18">
-        <v>1568503.2160000005</v>
+        <v>1764570.118</v>
       </c>
       <c r="K18">
-        <v>1568503.2160000005</v>
-      </c>
-      <c r="L18" s="2"/>
-      <c r="M18" s="2"/>
+        <v>1764570.118</v>
+      </c>
       <c r="N18">
         <v>2087933.4128</v>
       </c>
       <c r="O18">
-        <v>2087933.4128</v>
+        <v>1565949.05975</v>
       </c>
       <c r="P18">
-        <v>2087933.4128</v>
+        <v>2348925.09</v>
       </c>
       <c r="Q18">
-        <v>2087933.4128</v>
-      </c>
-      <c r="R18" s="2"/>
-      <c r="S18" s="2"/>
+        <v>2348925.09</v>
+      </c>
       <c r="T18">
-        <v>101686.74</v>
+        <v>379208.83</v>
       </c>
       <c r="U18">
-        <v>101686.74</v>
+        <v>426609.93375000003</v>
       </c>
       <c r="V18">
-        <v>101686.74</v>
+        <v>639914.9007</v>
       </c>
       <c r="W18">
-        <v>101686.74</v>
-      </c>
-      <c r="X18" s="2"/>
-      <c r="Y18" s="2"/>
+        <v>639914.9007</v>
+      </c>
     </row>
     <row r="19" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A19">
@@ -6159,58 +5625,50 @@
         <v>234515.065</v>
       </c>
       <c r="C19">
-        <v>234515.065</v>
+        <v>175886.29874999999</v>
       </c>
       <c r="D19">
-        <v>234515.065</v>
+        <v>263829.44819999998</v>
       </c>
       <c r="E19">
-        <v>234515.065</v>
-      </c>
-      <c r="F19" s="2"/>
-      <c r="G19" s="2"/>
+        <v>263829.44819999998</v>
+      </c>
       <c r="H19">
         <v>1565634.0028000006</v>
       </c>
       <c r="I19">
-        <v>1565634.0028000006</v>
+        <v>1174225.5022499999</v>
       </c>
       <c r="J19">
-        <v>1565634.0028000006</v>
+        <v>1761343.253</v>
       </c>
       <c r="K19">
-        <v>1565634.0028000006</v>
-      </c>
-      <c r="L19" s="2"/>
-      <c r="M19" s="2"/>
+        <v>1761343.253</v>
+      </c>
       <c r="N19">
         <v>2076927.41784</v>
       </c>
       <c r="O19">
-        <v>2076927.41784</v>
+        <v>1557695.5634999999</v>
       </c>
       <c r="P19">
-        <v>2076927.41784</v>
+        <v>2336543.3459999999</v>
       </c>
       <c r="Q19">
-        <v>2076927.41784</v>
-      </c>
-      <c r="R19" s="2"/>
-      <c r="S19" s="2"/>
+        <v>2336543.3459999999</v>
+      </c>
       <c r="T19">
-        <v>100176.44</v>
+        <v>371440.05</v>
       </c>
       <c r="U19">
-        <v>100176.44</v>
+        <v>417868.55625000002</v>
       </c>
       <c r="V19">
-        <v>100176.44</v>
+        <v>626802.83444999997</v>
       </c>
       <c r="W19">
-        <v>100176.44</v>
-      </c>
-      <c r="X19" s="2"/>
-      <c r="Y19" s="2"/>
+        <v>626802.83444999997</v>
+      </c>
     </row>
     <row r="20" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A20">
@@ -6220,58 +5678,50 @@
         <v>230944.68799999999</v>
       </c>
       <c r="C20">
-        <v>230944.68799999999</v>
+        <v>173208.516</v>
       </c>
       <c r="D20">
-        <v>230944.68799999999</v>
+        <v>259812.774</v>
       </c>
       <c r="E20">
-        <v>230944.68799999999</v>
-      </c>
-      <c r="F20" s="2"/>
-      <c r="G20" s="2"/>
+        <v>259812.774</v>
+      </c>
       <c r="H20">
         <v>1562764.7896000005</v>
       </c>
       <c r="I20">
-        <v>1562764.7896000005</v>
+        <v>1172073.5925</v>
       </c>
       <c r="J20">
-        <v>1562764.7896000005</v>
+        <v>1758116.3895</v>
       </c>
       <c r="K20">
-        <v>1562764.7896000005</v>
-      </c>
-      <c r="L20" s="2"/>
-      <c r="M20" s="2"/>
+        <v>1758116.3895</v>
+      </c>
       <c r="N20">
         <v>2065921.4228800002</v>
       </c>
       <c r="O20">
-        <v>2065921.4228800002</v>
+        <v>1549442.0672500001</v>
       </c>
       <c r="P20">
-        <v>2065921.4228800002</v>
+        <v>2324163.1005000002</v>
       </c>
       <c r="Q20">
-        <v>2065921.4228800002</v>
-      </c>
-      <c r="R20" s="2"/>
-      <c r="S20" s="2"/>
+        <v>2324163.1005000002</v>
+      </c>
       <c r="T20">
-        <v>98689.79</v>
+        <v>363834.24</v>
       </c>
       <c r="U20">
-        <v>98689.79</v>
+        <v>409307.52</v>
       </c>
       <c r="V20">
-        <v>98689.79</v>
+        <v>613961.28</v>
       </c>
       <c r="W20">
-        <v>98689.79</v>
-      </c>
-      <c r="X20" s="2"/>
-      <c r="Y20" s="2"/>
+        <v>613961.28</v>
+      </c>
     </row>
     <row r="21" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A21">
@@ -6281,58 +5731,50 @@
         <v>227422.96530000001</v>
       </c>
       <c r="C21">
-        <v>227422.96530000001</v>
+        <v>170567.223975</v>
       </c>
       <c r="D21">
-        <v>227422.96530000001</v>
+        <v>255850.83600000001</v>
       </c>
       <c r="E21">
-        <v>227422.96530000001</v>
-      </c>
-      <c r="F21" s="2"/>
-      <c r="G21" s="2"/>
+        <v>255850.83600000001</v>
+      </c>
       <c r="H21">
         <v>1559895.5764000006</v>
       </c>
       <c r="I21">
-        <v>1559895.5764000006</v>
+        <v>1169921.682</v>
       </c>
       <c r="J21">
-        <v>1559895.5764000006</v>
+        <v>1754889.523</v>
       </c>
       <c r="K21">
-        <v>1559895.5764000006</v>
-      </c>
-      <c r="L21" s="2"/>
-      <c r="M21" s="2"/>
+        <v>1754889.523</v>
+      </c>
       <c r="N21">
         <v>2054915.4279200002</v>
       </c>
       <c r="O21">
-        <v>2054915.4279200002</v>
+        <v>1541188.571</v>
       </c>
       <c r="P21">
-        <v>2054915.4279200002</v>
+        <v>2311782.8565000002</v>
       </c>
       <c r="Q21">
-        <v>2054915.4279200002</v>
-      </c>
-      <c r="R21" s="2"/>
-      <c r="S21" s="2"/>
+        <v>2311782.8565000002</v>
+      </c>
       <c r="T21">
-        <v>97226.44</v>
+        <v>356389.41</v>
       </c>
       <c r="U21">
-        <v>97226.44</v>
+        <v>400923.08624999999</v>
       </c>
       <c r="V21">
-        <v>97226.44</v>
+        <v>601384.62945000001</v>
       </c>
       <c r="W21">
-        <v>97226.44</v>
-      </c>
-      <c r="X21" s="2"/>
-      <c r="Y21" s="2"/>
+        <v>601384.62945000001</v>
+      </c>
     </row>
     <row r="22" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A22">
@@ -6342,66 +5784,62 @@
         <v>223948.88099999999</v>
       </c>
       <c r="C22">
-        <v>223948.88099999999</v>
+        <v>167961.66075000001</v>
       </c>
       <c r="D22">
-        <v>223948.88099999999</v>
+        <v>251942.49119999999</v>
       </c>
       <c r="E22">
-        <v>223948.88099999999</v>
+        <v>251942.49119999999</v>
       </c>
       <c r="F22">
-        <v>223948.88099999999</v>
-      </c>
-      <c r="G22" s="2"/>
+        <v>251942.49119999999</v>
+      </c>
       <c r="H22">
         <v>1557026.3632000005</v>
       </c>
       <c r="I22">
-        <v>1557026.3632000005</v>
+        <v>1167769.7722499999</v>
       </c>
       <c r="J22">
-        <v>1557026.3632000005</v>
+        <v>1751662.6580000001</v>
       </c>
       <c r="K22">
-        <v>1557026.3632000005</v>
+        <v>1751662.6580000001</v>
       </c>
       <c r="L22">
-        <v>1557026.3632000005</v>
-      </c>
-      <c r="M22" s="2"/>
+        <v>1751662.6580000001</v>
+      </c>
       <c r="N22">
         <v>2043909.4329600004</v>
       </c>
       <c r="O22">
-        <v>2043909.4329600004</v>
+        <v>1532935.0747499999</v>
       </c>
       <c r="P22">
-        <v>2043909.4329600004</v>
+        <v>2299402.6124999998</v>
       </c>
       <c r="Q22">
-        <v>2043909.4329600004</v>
+        <v>2299402.6124999998</v>
       </c>
       <c r="R22">
-        <v>2043909.4329600004</v>
-      </c>
-      <c r="S22" s="2"/>
+        <v>2299402.6124999998</v>
+      </c>
       <c r="T22">
-        <v>95786.05</v>
+        <v>349103.66</v>
       </c>
       <c r="U22">
-        <v>95786.05</v>
+        <v>392711.61749999999</v>
       </c>
       <c r="V22">
-        <v>95786.05</v>
+        <v>589067.42625000002</v>
       </c>
       <c r="W22">
-        <v>95786.05</v>
+        <v>589067.42625000002</v>
       </c>
       <c r="X22">
-        <v>95786.05</v>
-      </c>
-      <c r="Y22" s="2"/>
+        <v>589067.42625000002</v>
+      </c>
     </row>
     <row r="23" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A23">
@@ -6411,66 +5849,62 @@
         <v>220521.46350000001</v>
       </c>
       <c r="C23">
-        <v>220521.46350000001</v>
+        <v>165391.09770000001</v>
       </c>
       <c r="D23">
-        <v>220521.46350000001</v>
+        <v>248086.64655</v>
       </c>
       <c r="E23">
-        <v>220521.46350000001</v>
+        <v>248086.64655</v>
       </c>
       <c r="F23">
-        <v>220521.46350000001</v>
-      </c>
-      <c r="G23" s="2"/>
+        <v>248086.64655</v>
+      </c>
       <c r="H23">
         <v>1554157.1500000006</v>
       </c>
       <c r="I23">
-        <v>1554157.1500000006</v>
+        <v>1165617.8625</v>
       </c>
       <c r="J23">
-        <v>1554157.1500000006</v>
+        <v>1748435.7945000001</v>
       </c>
       <c r="K23">
-        <v>1554157.1500000006</v>
+        <v>1748435.7945000001</v>
       </c>
       <c r="L23">
-        <v>1554157.1500000006</v>
-      </c>
-      <c r="M23" s="2"/>
+        <v>1748435.7945000001</v>
+      </c>
       <c r="N23">
         <v>2032903.4380000005</v>
       </c>
       <c r="O23">
-        <v>2032903.4380000005</v>
+        <v>1524681.5785000001</v>
       </c>
       <c r="P23">
-        <v>2032903.4380000005</v>
+        <v>2287022.3684999999</v>
       </c>
       <c r="Q23">
-        <v>2032903.4380000005</v>
+        <v>2287022.3684999999</v>
       </c>
       <c r="R23">
-        <v>2032903.4380000005</v>
-      </c>
-      <c r="S23" s="2"/>
+        <v>2287022.3684999999</v>
+      </c>
       <c r="T23">
-        <v>94368.26</v>
+        <v>341975.1</v>
       </c>
       <c r="U23">
-        <v>94368.26</v>
+        <v>384669.48749999999</v>
       </c>
       <c r="V23">
-        <v>94368.26</v>
+        <v>577004.23124999995</v>
       </c>
       <c r="W23">
-        <v>94368.26</v>
+        <v>577004.23124999995</v>
       </c>
       <c r="X23">
-        <v>94368.26</v>
-      </c>
-      <c r="Y23" s="2"/>
+        <v>577004.23124999995</v>
+      </c>
     </row>
     <row r="24" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A24">
@@ -6480,66 +5914,62 @@
         <v>217139.74350000001</v>
       </c>
       <c r="C24">
-        <v>217139.74350000001</v>
+        <v>162854.80762499999</v>
       </c>
       <c r="D24">
-        <v>217139.74350000001</v>
+        <v>244282.2114</v>
       </c>
       <c r="E24">
-        <v>217139.74350000001</v>
+        <v>244282.2114</v>
       </c>
       <c r="F24">
-        <v>217139.74350000001</v>
-      </c>
-      <c r="G24" s="2"/>
+        <v>244282.2114</v>
+      </c>
       <c r="H24">
         <v>1551287.9368000007</v>
       </c>
       <c r="I24">
-        <v>1551287.9368000007</v>
+        <v>1163465.9527499999</v>
       </c>
       <c r="J24">
-        <v>1551287.9368000007</v>
+        <v>1745208.9295000001</v>
       </c>
       <c r="K24">
-        <v>1551287.9368000007</v>
+        <v>1745208.9295000001</v>
       </c>
       <c r="L24">
-        <v>1551287.9368000007</v>
-      </c>
-      <c r="M24" s="2"/>
+        <v>1745208.9295000001</v>
+      </c>
       <c r="N24">
         <v>2021897.4430400007</v>
       </c>
       <c r="O24">
-        <v>2021897.4430400007</v>
+        <v>1516428.08225</v>
       </c>
       <c r="P24">
-        <v>2021897.4430400007</v>
+        <v>2274642.1230000001</v>
       </c>
       <c r="Q24">
-        <v>2021897.4430400007</v>
+        <v>2274642.1230000001</v>
       </c>
       <c r="R24">
-        <v>2021897.4430400007</v>
-      </c>
-      <c r="S24" s="2"/>
+        <v>2274642.1230000001</v>
+      </c>
       <c r="T24">
-        <v>92972.74</v>
+        <v>334991.90000000002</v>
       </c>
       <c r="U24">
-        <v>92972.74</v>
+        <v>376793.88750000001</v>
       </c>
       <c r="V24">
-        <v>92972.74</v>
+        <v>565190.83125000005</v>
       </c>
       <c r="W24">
-        <v>92972.74</v>
+        <v>565190.83125000005</v>
       </c>
       <c r="X24">
-        <v>92972.74</v>
-      </c>
-      <c r="Y24" s="2"/>
+        <v>565190.83125000005</v>
+      </c>
     </row>
     <row r="25" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A25">
@@ -6549,66 +5979,62 @@
         <v>213802.75769999999</v>
       </c>
       <c r="C25">
-        <v>213802.75769999999</v>
+        <v>160352.06817499999</v>
       </c>
       <c r="D25">
-        <v>213802.75769999999</v>
+        <v>240528.1023</v>
       </c>
       <c r="E25">
-        <v>213802.75769999999</v>
+        <v>240528.1023</v>
       </c>
       <c r="F25">
-        <v>213802.75769999999</v>
-      </c>
-      <c r="G25" s="2"/>
+        <v>240528.1023</v>
+      </c>
       <c r="H25">
         <v>1548418.7236000006</v>
       </c>
       <c r="I25">
-        <v>1548418.7236000006</v>
+        <v>1161314.0430000001</v>
       </c>
       <c r="J25">
-        <v>1548418.7236000006</v>
+        <v>1741982.0645000001</v>
       </c>
       <c r="K25">
-        <v>1548418.7236000006</v>
+        <v>1741982.0645000001</v>
       </c>
       <c r="L25">
-        <v>1548418.7236000006</v>
-      </c>
-      <c r="M25" s="2"/>
+        <v>1741982.0645000001</v>
+      </c>
       <c r="N25">
         <v>2010891.4480800009</v>
       </c>
       <c r="O25">
-        <v>2010891.4480800009</v>
+        <v>1508174.5859999999</v>
       </c>
       <c r="P25">
-        <v>2010891.4480800009</v>
+        <v>2262261.8790000002</v>
       </c>
       <c r="Q25">
-        <v>2010891.4480800009</v>
+        <v>2262261.8790000002</v>
       </c>
       <c r="R25">
-        <v>2010891.4480800009</v>
-      </c>
-      <c r="S25" s="2"/>
+        <v>2262261.8790000002</v>
+      </c>
       <c r="T25">
-        <v>91599.15</v>
+        <v>328152.28999999998</v>
       </c>
       <c r="U25">
-        <v>91599.15</v>
+        <v>369081.32624999998</v>
       </c>
       <c r="V25">
-        <v>91599.15</v>
+        <v>553621.98944999999</v>
       </c>
       <c r="W25">
-        <v>91599.15</v>
+        <v>553621.98944999999</v>
       </c>
       <c r="X25">
-        <v>91599.15</v>
-      </c>
-      <c r="Y25" s="2"/>
+        <v>553621.98944999999</v>
+      </c>
     </row>
     <row r="26" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A26">
@@ -6618,66 +6044,62 @@
         <v>210509.61679999999</v>
       </c>
       <c r="C26">
-        <v>210509.61679999999</v>
+        <v>157882.2126</v>
       </c>
       <c r="D26">
-        <v>210509.61679999999</v>
+        <v>236823.31899999999</v>
       </c>
       <c r="E26">
-        <v>210509.61679999999</v>
+        <v>236823.31899999999</v>
       </c>
       <c r="F26">
-        <v>210509.61679999999</v>
-      </c>
-      <c r="G26" s="2"/>
+        <v>236823.31899999999</v>
+      </c>
       <c r="H26">
         <v>1545549.5104000007</v>
       </c>
       <c r="I26">
-        <v>1545549.5104000007</v>
+        <v>1159162.1329999999</v>
       </c>
       <c r="J26">
-        <v>1545549.5104000007</v>
+        <v>1738755.1995000001</v>
       </c>
       <c r="K26">
-        <v>1545549.5104000007</v>
+        <v>1738755.1995000001</v>
       </c>
       <c r="L26">
-        <v>1545549.5104000007</v>
-      </c>
-      <c r="M26" s="2"/>
+        <v>1738755.1995000001</v>
+      </c>
       <c r="N26">
         <v>1999885.4531200009</v>
       </c>
       <c r="O26">
-        <v>1999885.4531200009</v>
+        <v>1499921.08975</v>
       </c>
       <c r="P26">
-        <v>1999885.4531200009</v>
+        <v>2249881.6349999998</v>
       </c>
       <c r="Q26">
-        <v>1999885.4531200009</v>
+        <v>2249881.6349999998</v>
       </c>
       <c r="R26">
-        <v>1999885.4531200009</v>
-      </c>
-      <c r="S26" s="2"/>
+        <v>2249881.6349999998</v>
+      </c>
       <c r="T26">
-        <v>90247.16</v>
+        <v>321454.53999999998</v>
       </c>
       <c r="U26">
-        <v>90247.16</v>
+        <v>361528.65749999997</v>
       </c>
       <c r="V26">
-        <v>90247.16</v>
+        <v>542292.98624999996</v>
       </c>
       <c r="W26">
-        <v>90247.16</v>
+        <v>542292.98624999996</v>
       </c>
       <c r="X26">
-        <v>90247.16</v>
-      </c>
-      <c r="Y26" s="2"/>
+        <v>542292.98624999996</v>
+      </c>
     </row>
     <row r="27" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A27">
@@ -6687,73 +6109,73 @@
         <v>207259.3126</v>
       </c>
       <c r="C27">
-        <v>207259.3126</v>
+        <v>155444.48444999999</v>
       </c>
       <c r="D27">
-        <v>207259.3126</v>
+        <v>233166.72675</v>
       </c>
       <c r="E27">
-        <v>207259.3126</v>
+        <v>233166.72675</v>
       </c>
       <c r="F27">
-        <v>207259.3126</v>
+        <v>233166.72675</v>
       </c>
       <c r="G27">
-        <v>207259.3126</v>
+        <v>233166.72675</v>
       </c>
       <c r="H27">
         <v>1542680.2972000006</v>
       </c>
       <c r="I27">
-        <v>1542680.2972000006</v>
+        <v>1157010.223</v>
       </c>
       <c r="J27">
-        <v>1542680.2972000006</v>
+        <v>1735528.3345000001</v>
       </c>
       <c r="K27">
-        <v>1542680.2972000006</v>
+        <v>1735528.3345000001</v>
       </c>
       <c r="L27">
-        <v>1542680.2972000006</v>
+        <v>1735528.3345000001</v>
       </c>
       <c r="M27">
-        <v>1542680.2972000006</v>
+        <v>1735528.3345000001</v>
       </c>
       <c r="N27">
         <v>1988879.4581600011</v>
       </c>
       <c r="O27">
-        <v>1988879.4581600011</v>
+        <v>1491667.5935</v>
       </c>
       <c r="P27">
-        <v>1988879.4581600011</v>
+        <v>2237501.3909999998</v>
       </c>
       <c r="Q27">
-        <v>1988879.4581600011</v>
+        <v>2237501.3909999998</v>
       </c>
       <c r="R27">
-        <v>1988879.4581600011</v>
+        <v>2237501.3909999998</v>
       </c>
       <c r="S27">
-        <v>1988879.4581600011</v>
+        <v>2237501.3909999998</v>
       </c>
       <c r="T27">
-        <v>88916.45</v>
+        <v>314897</v>
       </c>
       <c r="U27">
-        <v>88916.45</v>
+        <v>354132.33750000002</v>
       </c>
       <c r="V27">
-        <v>88916.45</v>
+        <v>531198.50624999998</v>
       </c>
       <c r="W27">
-        <v>88916.45</v>
+        <v>531198.50624999998</v>
       </c>
       <c r="X27">
-        <v>88916.45</v>
+        <v>531198.50624999998</v>
       </c>
       <c r="Y27">
-        <v>88916.45</v>
+        <v>531198.50624999998</v>
       </c>
     </row>
     <row r="28" spans="1:25" x14ac:dyDescent="0.3">
@@ -6764,73 +6186,73 @@
         <v>204050.9535</v>
       </c>
       <c r="C28">
-        <v>204050.9535</v>
+        <v>153038.21512499999</v>
       </c>
       <c r="D28">
-        <v>204050.9535</v>
+        <v>229557.32264999999</v>
       </c>
       <c r="E28">
-        <v>204050.9535</v>
+        <v>229557.32264999999</v>
       </c>
       <c r="F28">
-        <v>204050.9535</v>
+        <v>229557.32264999999</v>
       </c>
       <c r="G28">
-        <v>204050.9535</v>
+        <v>229557.32264999999</v>
       </c>
       <c r="H28">
         <v>1539811.0840000003</v>
       </c>
       <c r="I28">
-        <v>1539811.0840000003</v>
+        <v>1154858.3130000001</v>
       </c>
       <c r="J28">
-        <v>1539811.0840000003</v>
+        <v>1732301.4694999999</v>
       </c>
       <c r="K28">
-        <v>1539811.0840000003</v>
+        <v>1732301.4694999999</v>
       </c>
       <c r="L28">
-        <v>1539811.0840000003</v>
+        <v>1732301.4694999999</v>
       </c>
       <c r="M28">
-        <v>1539811.0840000003</v>
+        <v>1732301.4694999999</v>
       </c>
       <c r="N28">
         <v>1977873.4631999999</v>
       </c>
       <c r="O28">
-        <v>1977873.4631999999</v>
+        <v>1483414.0972500001</v>
       </c>
       <c r="P28">
-        <v>1977873.4631999999</v>
+        <v>2225121.145</v>
       </c>
       <c r="Q28">
-        <v>1977873.4631999999</v>
+        <v>2225121.145</v>
       </c>
       <c r="R28">
-        <v>1977873.4631999999</v>
+        <v>2225121.145</v>
       </c>
       <c r="S28">
-        <v>1977873.4631999999</v>
+        <v>2225121.145</v>
       </c>
       <c r="T28">
-        <v>87606.7</v>
+        <v>308477.99</v>
       </c>
       <c r="U28">
-        <v>87606.7</v>
+        <v>346737.73875000002</v>
       </c>
       <c r="V28">
-        <v>87606.7</v>
+        <v>520106.60820000002</v>
       </c>
       <c r="W28">
-        <v>87606.7</v>
+        <v>520106.60820000002</v>
       </c>
       <c r="X28">
-        <v>87606.7</v>
+        <v>520106.60820000002</v>
       </c>
       <c r="Y28">
-        <v>87606.7</v>
+        <v>520106.60820000002</v>
       </c>
     </row>
   </sheetData>
@@ -8684,4 +8106,247 @@
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
   <drawing r:id="rId1"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{2F60D7FF-52FE-4E9C-8C92-EE039FC68DFA}">
+  <dimension ref="A1:G28"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetData>
+    <row r="1" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>68</v>
+      </c>
+      <c r="C1" t="s">
+        <v>69</v>
+      </c>
+      <c r="D1" t="s">
+        <v>70</v>
+      </c>
+      <c r="E1" t="s">
+        <v>71</v>
+      </c>
+      <c r="F1" t="s">
+        <v>72</v>
+      </c>
+      <c r="G1" t="s">
+        <v>73</v>
+      </c>
+    </row>
+    <row r="2" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A2">
+        <v>2024</v>
+      </c>
+      <c r="C2" s="2"/>
+      <c r="D2" s="2"/>
+      <c r="E2" s="2"/>
+      <c r="F2" s="2"/>
+      <c r="G2" s="2"/>
+    </row>
+    <row r="3" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A3">
+        <v>2025</v>
+      </c>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+      <c r="G3" s="2"/>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A4">
+        <v>2026</v>
+      </c>
+      <c r="C4" s="2"/>
+      <c r="D4" s="2"/>
+      <c r="E4" s="2"/>
+      <c r="F4" s="2"/>
+      <c r="G4" s="2"/>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A5">
+        <v>2027</v>
+      </c>
+      <c r="C5" s="2"/>
+      <c r="D5" s="2"/>
+      <c r="E5" s="2"/>
+      <c r="F5" s="2"/>
+      <c r="G5" s="2"/>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A6">
+        <v>2028</v>
+      </c>
+      <c r="C6" s="2"/>
+      <c r="D6" s="2"/>
+      <c r="E6" s="2"/>
+      <c r="F6" s="2"/>
+      <c r="G6" s="2"/>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A7">
+        <v>2029</v>
+      </c>
+      <c r="D7" s="2"/>
+      <c r="E7" s="2"/>
+      <c r="F7" s="2"/>
+      <c r="G7" s="2"/>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A8">
+        <v>2030</v>
+      </c>
+      <c r="D8" s="2"/>
+      <c r="E8" s="2"/>
+      <c r="F8" s="2"/>
+      <c r="G8" s="2"/>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A9">
+        <v>2031</v>
+      </c>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+      <c r="G9" s="2"/>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A10">
+        <v>2032</v>
+      </c>
+      <c r="D10" s="2"/>
+      <c r="E10" s="2"/>
+      <c r="F10" s="2"/>
+      <c r="G10" s="2"/>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A11">
+        <v>2033</v>
+      </c>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+      <c r="G11" s="2"/>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A12">
+        <v>2034</v>
+      </c>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+      <c r="G12" s="2"/>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A13">
+        <v>2035</v>
+      </c>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+      <c r="G13" s="2"/>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A14">
+        <v>2036</v>
+      </c>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+      <c r="G14" s="2"/>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A15">
+        <v>2037</v>
+      </c>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+      <c r="G15" s="2"/>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A16">
+        <v>2038</v>
+      </c>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+      <c r="G16" s="2"/>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A17">
+        <v>2039</v>
+      </c>
+      <c r="F17" s="2"/>
+      <c r="G17" s="2"/>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A18">
+        <v>2040</v>
+      </c>
+      <c r="F18" s="2"/>
+      <c r="G18" s="2"/>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A19">
+        <v>2041</v>
+      </c>
+      <c r="F19" s="2"/>
+      <c r="G19" s="2"/>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A20">
+        <v>2042</v>
+      </c>
+      <c r="F20" s="2"/>
+      <c r="G20" s="2"/>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A21">
+        <v>2043</v>
+      </c>
+      <c r="F21" s="2"/>
+      <c r="G21" s="2"/>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A22">
+        <v>2044</v>
+      </c>
+      <c r="G22" s="2"/>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A23">
+        <v>2045</v>
+      </c>
+      <c r="G23" s="2"/>
+    </row>
+    <row r="24" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A24">
+        <v>2046</v>
+      </c>
+      <c r="G24" s="2"/>
+    </row>
+    <row r="25" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A25">
+        <v>2047</v>
+      </c>
+      <c r="G25" s="2"/>
+    </row>
+    <row r="26" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A26">
+        <v>2048</v>
+      </c>
+      <c r="G26" s="2"/>
+    </row>
+    <row r="27" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A27">
+        <v>2049</v>
+      </c>
+    </row>
+    <row r="28" spans="1:7" x14ac:dyDescent="0.3">
+      <c r="A28">
+        <v>2050</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>